<commit_message>
Excel formatori DE v1: 9 freelance + 5 istituzioni + 7 concorrenti — 3 sheet formattati
</commit_message>
<xml_diff>
--- a/data/trainers/ErasmusDidactica_FORMATORI_DE_v1.xlsx
+++ b/data/trainers/ErasmusDidactica_FORMATORI_DE_v1.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONCORRENTI" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FORMATORI_FREELANCE'!$A$2:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FORMATORI_FREELANCE'!$A$2:$L$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ISTITUZIONI_PUBBLICHE'!$A$2:$L$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CONCORRENTI'!$A$2:$L$9</definedName>
   </definedNames>
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,7 +33,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00003366"/>
+      <color rgb="00FFFFFF"/>
       <sz val="16"/>
     </font>
     <font>
@@ -41,8 +41,11 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -69,8 +72,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E0E0E0"/>
-        <bgColor rgb="00E0E0E0"/>
+        <fgColor rgb="00404040"/>
+        <bgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
+        <bgColor rgb="00E8E8E8"/>
       </patternFill>
     </fill>
   </fills>
@@ -92,21 +101,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,31 +489,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ErasmusDidactica — FORMATORI_FREELANCE (7 record)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>ErasmusDidactica — FORMATORI_FREELANCE (9 record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ID</t>
@@ -560,7 +575,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="40" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>DE-T002</t>
@@ -618,7 +633,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="40" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>DE-T003</t>
@@ -672,7 +687,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="40" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>DE-T007</t>
@@ -730,7 +745,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>DE-T008</t>
@@ -788,7 +803,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="40" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>DE-T015</t>
@@ -846,7 +861,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="40" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>DE-T018</t>
@@ -896,7 +911,7 @@
       </c>
       <c r="L8" s="3" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="40" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>DE-T019</t>
@@ -946,8 +961,128 @@
       </c>
       <c r="L9" s="3" t="n"/>
     </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>DE-T020</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Ulrich Engelke</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>MediaPage / lehren-mit-ki.de</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>KI/AI für Lehrkräfte / ChatGPT in der Schule / Didattica digitale</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Augsburg</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>info@lehren-mit-ki.de</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>https://lehren-mit-ki.de</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ulrich-engelke-9442075b/</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Co-trainer: Barbara Engelke (docente Gymnasium). 2 libri: ChatGPT &amp; Co. in der Schule. VAT DE151171097. Tel +49 821 9000-260. Workshop max 8 pers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>DE-T021</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Barbara Engelke</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>MediaPage / lehren-mit-ki.de</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>KI im Unterricht / Deutsch / Religion / Gymnasium-Didaktik</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Augsburg</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>info@lehren-mit-ki.de</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>https://lehren-mit-ki.de</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Gymnasiallehrerin Deutsch+Religion. Fachleitung Deutsch. Co-autrice 2 libri KI. Erfahrung Schulpraxis.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L9"/>
+  <autoFilter ref="A2:L11"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -964,28 +1099,28 @@
   <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ErasmusDidactica — ISTITUZIONI_PUBBLICHE (5 record)</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ID</t>
@@ -1047,7 +1182,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="40" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>DE-T009</t>
@@ -1097,26 +1232,26 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="40" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>DE-T011</t>
+          <t>DE-T010</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Pädagogisches Institut München (PI)</t>
+          <t>Institut für Lehrerfortbildung (ILF)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Istituzione pubblica</t>
+          <t>Istituzione</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Internationale Bildungskooperationen / Erasmus+</t>
+          <t>Religionspädagogik / cattolica</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1126,13 +1261,13 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>München</t>
+          <t>Gars am Inn</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>https://www.pi-muenchen.de</t>
+          <t>https://www.gars-ilf.de</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
@@ -1143,20 +1278,20 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Supporto Erasmus+ per scuole Monaco. Fachbereich IBK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Formazione insegnanti religione cattolica Bayern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>DE-T016</t>
+          <t>DE-T011</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Bildung-International Hamburg</t>
+          <t>Pädagogisches Institut München (PI)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1166,7 +1301,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Erasmus+ Fortbildung Lehrkräfte Ausland</t>
+          <t>Internationale Bildungskooperationen / Erasmus+</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -1176,13 +1311,13 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>München</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://bildung-international.hamburg.de</t>
+          <t>https://www.pi-muenchen.de</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
@@ -1193,20 +1328,20 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Behörde für Schule und Berufsbildung. Supporto Erasmus+ per scuole Hamburg.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>Supporto Erasmus+ per scuole Monaco. Fachbereich IBK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>DE-T017</t>
+          <t>DE-T016</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Erasmus@ISB Bayern</t>
+          <t>Bildung-International Hamburg</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1216,7 +1351,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Erasmus+ Schulbildung Bayern</t>
+          <t>Erasmus+ Fortbildung Lehrkräfte Ausland</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -1226,13 +1361,13 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>München</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>https://www.erasmusplus.bayern.de</t>
+          <t>https://bildung-international.hamburg.de</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
@@ -1243,30 +1378,30 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>ISB = Staatsinstitut für Schulqualität. Koordina Erasmus+ per Bayern.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>Behörde für Schule und Berufsbildung. Supporto Erasmus+ per scuole Hamburg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>DE-T010</t>
+          <t>DE-T017</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Institut für Lehrerfortbildung (ILF)</t>
+          <t>Erasmus@ISB Bayern</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Istituzione</t>
+          <t>Istituzione pubblica</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Religionspädagogik / cattolica</t>
+          <t>Erasmus+ Schulbildung Bayern</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1276,13 +1411,13 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Gars am Inn</t>
+          <t>München</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>https://www.gars-ilf.de</t>
+          <t>https://www.erasmusplus.bayern.de</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
@@ -1293,7 +1428,7 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Formazione insegnanti religione cattolica Bayern.</t>
+          <t>ISB = Staatsinstitut für Schulqualität. Koordina Erasmus+ per Bayern.</t>
         </is>
       </c>
     </row>
@@ -1315,434 +1450,434 @@
   <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>ErasmusDidactica — CONCORRENTI (7 record)</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Organizzazione</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Specializzazione</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Citta</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>Sito_Web</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>LinkedIn_URL</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>Fonte_URL</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>DE-T001</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>ZORYA Limited</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Provider KA1</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Stress management / Zeitmanagement / Gesundheit / Digitale Lösungen</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Cipro (sede legale)</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>contact@erasmus-fortbildung.com</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>https://www.erasmus-fortbildung.com</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr"/>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr"/>
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Web</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>OID: E10369220. 850+ partecipanti. Rating 4.9/5. Tel: +357 97949119. Registrato ORS EU.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>DE-T004</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Erasmus Learning Academy (ELA)</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Provider KA1</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Classroom Management / ICT-AI / Inclusion / Innovation / Well-being</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Bologna + Palermo + Berlin</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>info@erasmuslearningacademy.eu</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>https://erasmustrainingcourses.com</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr"/>
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>Web</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>OID: E10221762 (IT) + E10303586 (ES). 10000+ docenti. ISO 9001. Tel Bologna: +39 380 8698725.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>DE-T005</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>EBB Europass Berlin Beratungsbüro GmbH</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Provider KA1</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>STEAM / PBL / 21st century skills / Classroom management / Bullying prevention</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Berlin</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr"/>
+      <c r="I5" s="7" t="inlineStr">
         <is>
           <t>https://www.teacheracademy.eu/courses-location/berlin/</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr"/>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="J5" s="7" t="inlineStr"/>
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>Web</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>OID: E10233216. Teacher Academy Berlin. Corsi 1-2 settimane. Topics: innovazione didattica.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>DE-T006</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Europass Teacher Academy (Network)</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Provider KA1</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>400+ corsi KA1 tutte le materie</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Firenze + 30 sedi</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr"/>
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>https://www.teacheracademy.eu</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="J6" s="7" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>Web</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L6" s="7" t="inlineStr">
         <is>
           <t>Più grande provider Erasmus+ KA1 Europa. Sedi in 30+ città.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>DE-T012</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Educat Academy</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Provider KA1</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>STEM / Digitale / Inclusione</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Cipro + Grecia + Lituania</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>https://educat.academy</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr"/>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr"/>
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>Web</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
         <is>
           <t>OID: E10339100. Docenti da DE/PL/FR/ES/IT.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>DE-T013</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr"/>
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>iTEACH ITL-INSTITUTE</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Provider KA1</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>KA1 Kurse / Methodik</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>https://www.itl-institute.com</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr"/>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>Web</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr">
         <is>
           <t>~100 corsi erogati.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>DE-T014</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>ARAXÁ Edu</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Provider KA1</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Teacher development / Training delivery</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>https://araxaedu.com</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>Web</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>Corsi registrati su ESEP.</t>
         </is>

</xml_diff>

<commit_message>
TASK 3+4: 31 formatori DE (17 freelance + 7 istituzioni + 7 concorrenti) + template outreach DE 3 varianti
</commit_message>
<xml_diff>
--- a/data/trainers/ErasmusDidactica_FORMATORI_DE_v1.xlsx
+++ b/data/trainers/ErasmusDidactica_FORMATORI_DE_v1.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONCORRENTI" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FORMATORI_FREELANCE'!$A$2:$L$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ISTITUZIONI_PUBBLICHE'!$A$2:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FORMATORI_FREELANCE'!$A$2:$L$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ISTITUZIONI_PUBBLICHE'!$A$2:$L$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CONCORRENTI'!$A$2:$L$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,16 +489,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
@@ -506,14 +506,14 @@
     <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ErasmusDidactica — FORMATORI_FREELANCE (9 record)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="25" customHeight="1">
+          <t>ErasmusDidactica — FORMATORI_FREELANCE (17 record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ID</t>
@@ -575,7 +575,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="40" customHeight="1">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>DE-T002</t>
@@ -633,7 +633,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>DE-T003</t>
@@ -687,7 +687,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>DE-T007</t>
@@ -745,7 +745,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>DE-T008</t>
@@ -803,7 +803,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>DE-T015</t>
@@ -861,7 +861,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>DE-T018</t>
@@ -909,9 +909,9 @@
           <t>Freelance trainer specializzata progetti Erasmus+.</t>
         </is>
       </c>
-      <c r="L8" s="3" t="n"/>
-    </row>
-    <row r="9" ht="40" customHeight="1">
+      <c r="L8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>DE-T019</t>
@@ -959,9 +959,9 @@
           <t>10 anni esperienza. Coaching + e-learning + pedagogia. Basata in DE.</t>
         </is>
       </c>
-      <c r="L9" s="3" t="n"/>
-    </row>
-    <row r="10" ht="40" customHeight="1">
+      <c r="L9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>DE-T020</t>
@@ -974,7 +974,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>MediaPage / lehren-mit-ki.de</t>
+          <t>MediaPage / lehren-mit-ki.de / der-ki-trainer.de</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -1019,11 +1019,11 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Co-trainer: Barbara Engelke (docente Gymnasium). 2 libri: ChatGPT &amp; Co. in der Schule. VAT DE151171097. Tel +49 821 9000-260. Workshop max 8 pers.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
+          <t>2 libri: ChatGPT &amp; Co. in der Schule. VAT DE151171097. Tel +49 821 9000-260. Workshop max 8 pers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>DE-T021</t>
@@ -1077,12 +1077,460 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>Gymnasiallehrerin Deutsch+Religion. Fachleitung Deutsch. Co-autrice 2 libri KI. Erfahrung Schulpraxis.</t>
+          <t>Gymnasiallehrerin Deutsch+Religion. Fachleitung. Co-autrice 2 libri KI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>DE-T022</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Diana Knodel</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>fobizz / 101skills GmbH</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Digitale Kompetenzen Lehrkräfte / KI-Zusatzqualifikation / EdTech</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>kontakt@fobizz.com</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>https://fobizz.com</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Co-Gründerin fobizz. Deutschlands größte Fortbildungsplattform Lehrer. Tel +49 40 743 04189. HRB 152465 Hamburg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>DE-T023</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Frederik Dietz</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>fobizz / 101skills GmbH</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Digitale Bildung / EdTech / KI für Lehrkräfte</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>kontakt@fobizz.com</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>https://fobizz.com</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Co-Gründer fobizz. Managing Partner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>DE-T024</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Steffen Schneider</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>KI macht Schule gGmbH</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>KI-Workshops Schulen / Machine Learning für Lehrkräfte</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Tübingen</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>info@ki-macht-schule.de</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>https://ki-macht-schule.de</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Founder+CEO. Team 100+ Trainer. Sitz: Maria-von-Linden-Str. 6, 72076 Tübingen. HRB 781709.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>DE-T025</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sarah Schönbrodt</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>KI macht Schule gGmbH</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Kursentwicklung / Didaktik / KI in Bildung</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Tübingen</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>info@ki-macht-schule.de</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>https://ki-macht-schule.de</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Co-CEO. Verantwortlich Kursentwicklung &amp; Didaktik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>DE-T026</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Sven Walter</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Baden-Württemberg Stiftung</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Istituzione</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Inklusion / Schulbegleitung / Fortbildung</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>walter@bwstiftung.de</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bwstiftung.de</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Ansprechpartner Inklusion. Tel +49 711 248 476-24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>DE-T027</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Ines Homburg</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Lehrkräfteakademie Hessen</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Istituzione</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Inklusion Lehrerausbildung / Fortbildung Hessen</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Ines.Homburg@schule.hessen.de</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>https://lehrkraefteakademie.hessen.de</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Beratung Inklusion in Lehrkräfteausbildung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>DE-T028</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Franziska Drauz</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Zukunft Digitale Bildung gGmbH</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Digitale Bildung / Partnermanagement / Lehrerfortbildung</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>https://zukunft-digitale-bildung.de</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr"/>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Geschäftsleitung Partnermanagement. Sitz: Ahlbeckerstr. 12, 10437 Berlin. HRB 219501.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>DE-T029</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>DigitalErleben</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Freelance</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>KI Tools / Fortbildungen vor Ort / IServ / Office365 / paddy</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>https://digitalerleben.de</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr"/>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Team giovani Trainer. Tel +49 176 42962392. 400+ Fortbildungen. Viene a scuola.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:L11"/>
+  <autoFilter ref="A2:L19"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -1096,16 +1544,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
@@ -1113,14 +1561,14 @@
     <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ErasmusDidactica — ISTITUZIONI_PUBBLICHE (5 record)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="25" customHeight="1">
+          <t>ErasmusDidactica — ISTITUZIONI_PUBBLICHE (7 record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ID</t>
@@ -1182,7 +1630,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="40" customHeight="1">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>DE-T009</t>
@@ -1232,7 +1680,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>DE-T010</t>
@@ -1282,7 +1730,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>DE-T011</t>
@@ -1332,7 +1780,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>DE-T016</t>
@@ -1382,7 +1830,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>DE-T017</t>
@@ -1432,8 +1880,112 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>DE-T030</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Science on Stage Deutschland e.V.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Istituzione</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>MINT Lehrerfortbildung / von Lehrkräften für Lehrkräfte</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>info@science-on-stage.de</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.science-on-stage.de</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Am Borsigturm 15, 13507 Berlin. Tel +49 30 400067-40. Trainer = MINT-Lehrkräfte mit Festival-Erfahrung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>DE-T031</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Stiftung Kinder forschen</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Istituzione</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>MINT Fortbildung / Grundschule + Sekundarstufe I</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.stiftung-kinder-forschen.de</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Netzwerk-Trainer mit pädagogischem oder MINT-Hintergrund. Regionaler Einsatz.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:L7"/>
+  <autoFilter ref="A2:L9"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -1453,10 +2005,10 @@
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
@@ -1464,14 +2016,14 @@
     <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>ErasmusDidactica — CONCORRENTI (7 record)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>ID</t>
@@ -1533,7 +2085,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="40" customHeight="1">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>DE-T001</t>
@@ -1587,7 +2139,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>DE-T004</t>
@@ -1641,7 +2193,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>DE-T005</t>
@@ -1691,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>DE-T006</t>
@@ -1741,7 +2293,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>DE-T012</t>
@@ -1791,7 +2343,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>DE-T013</t>
@@ -1837,7 +2389,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>DE-T014</t>

</xml_diff>